<commit_message>
Fix Red Fight Requirements - There was no logical requirement to have Fire/Electric/Charge in order to deal with the critters in phase 2...whoops.
</commit_message>
<xml_diff>
--- a/worlds/spyro_aht/setup/Gem Research.xlsx
+++ b/worlds/spyro_aht/setup/Gem Research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8F4A0C-EC1E-4D09-8506-301519FAFF40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D95D44-01AB-4806-9A15-D0C2C463CF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2042,9 +2042,6 @@
     <t>armored chests by dragon egg via cannon/and baskets by dragon egg</t>
   </si>
   <si>
-    <t>on the ground/meatl chests/headbash chests</t>
-  </si>
-  <si>
     <t>on the ground/baskets/and metal chests after electric platform</t>
   </si>
   <si>
@@ -2349,6 +2346,9 @@
   </si>
   <si>
     <t>horn diveable barrels/crates</t>
+  </si>
+  <si>
+    <t>on the ground/metal chests/headbash chests</t>
   </si>
 </sst>
 </file>
@@ -2927,7 +2927,7 @@
         <v>395</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>20</v>
@@ -2941,7 +2941,7 @@
         <v>360</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>20</v>
@@ -3941,7 +3941,7 @@
         <v>1003</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>20</v>
@@ -3955,7 +3955,7 @@
         <v>928</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>20</v>
@@ -4436,7 +4436,7 @@
         <v>675</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>20</v>
@@ -4450,7 +4450,7 @@
         <v>700</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>20</v>
@@ -5834,7 +5834,7 @@
         <v>755</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D223" s="3" t="s">
         <v>20</v>
@@ -5848,7 +5848,7 @@
         <v>1435</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D224" s="3" t="s">
         <v>20</v>
@@ -6651,7 +6651,7 @@
         <v>200</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D282" s="3" t="s">
         <v>20</v>
@@ -6665,7 +6665,7 @@
         <v>200</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D283" s="3" t="s">
         <v>20</v>
@@ -7272,7 +7272,7 @@
         <v>900</v>
       </c>
       <c r="C327" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D327" s="3" t="s">
         <v>20</v>
@@ -7286,7 +7286,7 @@
         <v>800</v>
       </c>
       <c r="C328" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D328" s="3" t="s">
         <v>20</v>
@@ -7721,7 +7721,7 @@
         <v>50</v>
       </c>
       <c r="C359" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D359" s="3" t="s">
         <v>35</v>
@@ -8132,7 +8132,7 @@
         <v>1906</v>
       </c>
       <c r="C389" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D389" s="3" t="s">
         <v>20</v>
@@ -8146,7 +8146,7 @@
         <v>1956</v>
       </c>
       <c r="C390" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D390" s="3" t="s">
         <v>20</v>
@@ -8219,7 +8219,7 @@
         <v>50</v>
       </c>
       <c r="C395" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D395" s="3" t="s">
         <v>214</v>
@@ -8905,7 +8905,7 @@
     </row>
     <row r="445" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A445" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B445" s="1">
         <v>110</v>
@@ -8919,7 +8919,7 @@
     </row>
     <row r="446" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A446" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B446" s="1">
         <v>156</v>
@@ -8936,7 +8936,7 @@
     </row>
     <row r="447" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A447" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B447" s="1">
         <v>400</v>
@@ -8950,7 +8950,7 @@
     </row>
     <row r="448" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A448" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B448" s="1">
         <v>500</v>
@@ -8964,7 +8964,7 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A449" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B449" s="1">
         <v>400</v>
@@ -8978,7 +8978,7 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A450" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B450" s="1">
         <v>60</v>
@@ -8992,7 +8992,7 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A451" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B451" s="1">
         <v>100</v>
@@ -9006,7 +9006,7 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A452" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B452" s="1">
         <v>1000</v>
@@ -9020,7 +9020,7 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A453" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B453" s="1">
         <v>450</v>
@@ -9034,7 +9034,7 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A454" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B454" s="1">
         <v>50</v>
@@ -9048,13 +9048,13 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A455" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B455" s="1">
         <v>950</v>
       </c>
       <c r="C455" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D455" s="3" t="s">
         <v>20</v>
@@ -9062,13 +9062,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A456" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B456" s="1">
         <v>900</v>
       </c>
       <c r="C456" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D456" s="3" t="s">
         <v>20</v>
@@ -9076,7 +9076,7 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A457" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B457" s="1">
         <v>200</v>
@@ -9703,7 +9703,7 @@
         <v>800</v>
       </c>
       <c r="C502" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="D502" s="3" t="s">
         <v>20</v>
@@ -9717,7 +9717,7 @@
         <v>830</v>
       </c>
       <c r="C503" s="1" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D503" s="3" t="s">
         <v>20</v>
@@ -10383,7 +10383,7 @@
         <v>270</v>
       </c>
       <c r="C551" s="1" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D551" s="3" t="s">
         <v>20</v>
@@ -10808,7 +10808,7 @@
         <v>443</v>
       </c>
       <c r="C582" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="D582" s="3" t="s">
         <v>20</v>
@@ -10822,7 +10822,7 @@
         <v>443</v>
       </c>
       <c r="C583" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D583" s="3" t="s">
         <v>20</v>
@@ -10836,7 +10836,7 @@
         <v>50</v>
       </c>
       <c r="C584" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D584" s="3" t="s">
         <v>20</v>
@@ -10928,13 +10928,13 @@
     </row>
     <row r="591" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A591" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B591" s="1">
         <v>50</v>
       </c>
       <c r="C591" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="D591" s="3" t="s">
         <v>20</v>
@@ -10942,7 +10942,7 @@
     </row>
     <row r="592" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A592" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B592" s="1">
         <v>25</v>
@@ -10956,7 +10956,7 @@
     </row>
     <row r="593" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A593" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B593" s="1">
         <v>130</v>
@@ -10970,7 +10970,7 @@
     </row>
     <row r="594" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A594" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B594" s="1">
         <v>55</v>
@@ -10984,7 +10984,7 @@
     </row>
     <row r="595" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A595" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B595" s="1">
         <v>50</v>
@@ -12216,7 +12216,7 @@
         <v>1100</v>
       </c>
       <c r="C683" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D683" s="3" t="s">
         <v>20</v>
@@ -12230,7 +12230,7 @@
         <v>900</v>
       </c>
       <c r="C684" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D684" s="3" t="s">
         <v>20</v>
@@ -12425,7 +12425,7 @@
     </row>
     <row r="699" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A699" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B699" s="1">
         <v>20</v>
@@ -12439,7 +12439,7 @@
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A700" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B700" s="1">
         <v>25</v>
@@ -12453,7 +12453,7 @@
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A701" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B701" s="1">
         <v>100</v>
@@ -12467,7 +12467,7 @@
     </row>
     <row r="702" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A702" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B702" s="1">
         <v>75</v>
@@ -12481,7 +12481,7 @@
     </row>
     <row r="703" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A703" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B703" s="1">
         <v>40</v>
@@ -12495,7 +12495,7 @@
     </row>
     <row r="704" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A704" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B704" s="1">
         <v>150</v>
@@ -12509,7 +12509,7 @@
     </row>
     <row r="705" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A705" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B705" s="1">
         <v>125</v>
@@ -12523,7 +12523,7 @@
     </row>
     <row r="706" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A706" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B706" s="1">
         <v>60</v>
@@ -12537,7 +12537,7 @@
     </row>
     <row r="707" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A707" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B707" s="1">
         <v>50</v>
@@ -12551,7 +12551,7 @@
     </row>
     <row r="708" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A708" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B708" s="1">
         <v>350</v>
@@ -12764,7 +12764,7 @@
     </row>
     <row r="723" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A723" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B723" s="1">
         <v>200</v>
@@ -12778,7 +12778,7 @@
     </row>
     <row r="724" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A724" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B724" s="1">
         <v>100</v>
@@ -12792,7 +12792,7 @@
     </row>
     <row r="725" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A725" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B725" s="1">
         <v>100</v>
@@ -12806,7 +12806,7 @@
     </row>
     <row r="726" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A726" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B726" s="1">
         <v>90</v>
@@ -12820,13 +12820,13 @@
     </row>
     <row r="727" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A727" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B727" s="1">
         <v>5240</v>
       </c>
       <c r="C727" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D727" s="3" t="s">
         <v>20</v>
@@ -12834,13 +12834,13 @@
     </row>
     <row r="728" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A728" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B728" s="1">
         <v>6980</v>
       </c>
       <c r="C728" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D728" s="3" t="s">
         <v>20</v>
@@ -12848,7 +12848,7 @@
     </row>
     <row r="729" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A729" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B729" s="1">
         <v>40</v>
@@ -12862,7 +12862,7 @@
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A730" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B730" s="1">
         <v>175</v>
@@ -12876,13 +12876,13 @@
     </row>
     <row r="731" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A731" s="1" t="s">
+        <v>666</v>
+      </c>
+      <c r="B731" s="1">
+        <v>20</v>
+      </c>
+      <c r="C731" s="1" t="s">
         <v>667</v>
-      </c>
-      <c r="B731" s="1">
-        <v>20</v>
-      </c>
-      <c r="C731" s="1" t="s">
-        <v>668</v>
       </c>
       <c r="D731" s="3" t="s">
         <v>395</v>
@@ -12890,7 +12890,7 @@
     </row>
     <row r="732" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A732" s="1" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B732" s="1">
         <v>50</v>
@@ -13072,7 +13072,7 @@
     </row>
     <row r="745" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A745" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B745" s="1">
         <v>75</v>
@@ -13086,7 +13086,7 @@
     </row>
     <row r="746" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A746" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B746" s="1">
         <v>20</v>
@@ -13100,7 +13100,7 @@
     </row>
     <row r="747" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A747" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B747" s="1">
         <v>20</v>
@@ -13114,7 +13114,7 @@
     </row>
     <row r="748" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A748" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B748" s="1">
         <v>50</v>
@@ -13128,7 +13128,7 @@
     </row>
     <row r="749" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A749" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B749" s="1">
         <v>100</v>
@@ -13142,7 +13142,7 @@
     </row>
     <row r="750" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A750" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B750" s="1">
         <v>25</v>
@@ -14130,7 +14130,7 @@
     </row>
     <row r="823" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A823" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B823" s="1">
         <v>16353</v>
@@ -14138,7 +14138,7 @@
     </row>
     <row r="824" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A824" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B824" s="1">
         <f>B821-B822-B823</f>
@@ -14290,7 +14290,7 @@
         <v>395</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>20</v>
@@ -14304,7 +14304,7 @@
         <v>360</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>20</v>
@@ -15014,7 +15014,7 @@
         <v>1003</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>20</v>
@@ -15028,7 +15028,7 @@
         <v>928</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>20</v>
@@ -15372,7 +15372,7 @@
         <v>675</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>20</v>
@@ -15386,7 +15386,7 @@
         <v>700</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>20</v>
@@ -16123,7 +16123,7 @@
         <v>525</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>581</v>
+        <v>683</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>20</v>
@@ -16193,7 +16193,7 @@
         <v>388</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>220</v>
@@ -16264,7 +16264,7 @@
         <v>115</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>48</v>
@@ -16362,7 +16362,7 @@
         <v>120</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>48</v>
@@ -16390,7 +16390,7 @@
         <v>755</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>20</v>
@@ -16404,7 +16404,7 @@
         <v>1435</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>20</v>
@@ -16593,7 +16593,7 @@
         <v>180</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D176" s="3" t="s">
         <v>20</v>
@@ -16776,7 +16776,7 @@
         <v>755</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D189" s="3" t="s">
         <v>20</v>
@@ -16861,7 +16861,7 @@
         <v>505</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D195" s="3" t="s">
         <v>20</v>
@@ -16889,7 +16889,7 @@
         <v>200</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D197" s="3" t="s">
         <v>20</v>
@@ -16903,7 +16903,7 @@
         <v>200</v>
       </c>
       <c r="C198" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>20</v>
@@ -16932,7 +16932,7 @@
         <v>410</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>20</v>
@@ -17008,7 +17008,7 @@
         <v>125</v>
       </c>
       <c r="C206" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D206" s="3" t="s">
         <v>48</v>
@@ -17121,7 +17121,7 @@
         <v>397</v>
       </c>
       <c r="C214" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D214" s="3" t="s">
         <v>66</v>
@@ -17387,7 +17387,7 @@
         <v>900</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D233" s="3" t="s">
         <v>20</v>
@@ -17401,7 +17401,7 @@
         <v>800</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D234" s="3" t="s">
         <v>20</v>
@@ -17529,7 +17529,7 @@
         <v>606</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D243" s="3" t="s">
         <v>20</v>
@@ -17557,7 +17557,7 @@
         <v>235</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D245" s="3" t="s">
         <v>20</v>
@@ -17572,7 +17572,7 @@
         <v>513</v>
       </c>
       <c r="C246" s="1" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D246" s="3" t="s">
         <v>20</v>
@@ -17670,7 +17670,7 @@
         <v>50</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="D253" s="3" t="s">
         <v>35</v>
@@ -17713,7 +17713,7 @@
         <v>250</v>
       </c>
       <c r="C256" s="1" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D256" s="3" t="s">
         <v>20</v>
@@ -17728,7 +17728,7 @@
         <v>342</v>
       </c>
       <c r="C257" s="1" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D257" s="3" t="s">
         <v>20</v>
@@ -17775,7 +17775,7 @@
         <v>100</v>
       </c>
       <c r="C261" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D261" s="3" t="s">
         <v>20</v>
@@ -17873,7 +17873,7 @@
         <v>145</v>
       </c>
       <c r="C268" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D268" s="3" t="s">
         <v>48</v>
@@ -17902,7 +17902,7 @@
         <v>1016</v>
       </c>
       <c r="C270" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D270" s="3" t="s">
         <v>20</v>
@@ -17916,7 +17916,7 @@
         <v>1906</v>
       </c>
       <c r="C271" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D271" s="3" t="s">
         <v>20</v>
@@ -17930,7 +17930,7 @@
         <v>1956</v>
       </c>
       <c r="C272" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D272" s="3" t="s">
         <v>20</v>
@@ -17986,7 +17986,7 @@
         <v>50</v>
       </c>
       <c r="C276" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D276" s="3" t="s">
         <v>214</v>
@@ -18056,7 +18056,7 @@
         <v>141</v>
       </c>
       <c r="C281" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D281" s="3" t="s">
         <v>22</v>
@@ -18070,7 +18070,7 @@
         <v>571</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D282" s="3" t="s">
         <v>20</v>
@@ -18226,7 +18226,7 @@
         <v>1166</v>
       </c>
       <c r="C293" s="1" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D293" s="3" t="s">
         <v>20</v>
@@ -18464,7 +18464,7 @@
         <v>160</v>
       </c>
       <c r="C310" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="D310" s="3" t="s">
         <v>297</v>
@@ -18491,7 +18491,7 @@
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A313" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B313" s="1">
         <v>110</v>
@@ -18505,13 +18505,13 @@
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A314" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B314" s="1">
         <v>656</v>
       </c>
       <c r="C314" s="1" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D314" s="3" t="s">
         <v>20</v>
@@ -18519,7 +18519,7 @@
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A315" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B315" s="1">
         <v>1060</v>
@@ -18533,7 +18533,7 @@
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A316" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B316" s="1">
         <v>400</v>
@@ -18547,7 +18547,7 @@
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A317" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B317" s="1">
         <v>1000</v>
@@ -18561,13 +18561,13 @@
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A318" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B318" s="1">
         <v>200</v>
       </c>
       <c r="C318" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D318" s="3" t="s">
         <v>20</v>
@@ -18575,13 +18575,13 @@
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A319" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B319" s="1">
         <v>950</v>
       </c>
       <c r="C319" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D319" s="3" t="s">
         <v>20</v>
@@ -18589,13 +18589,13 @@
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A320" s="1" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B320" s="1">
         <v>900</v>
       </c>
       <c r="C320" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D320" s="3" t="s">
         <v>20</v>
@@ -18782,7 +18782,7 @@
         <v>40</v>
       </c>
       <c r="C334" s="1" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D334" s="3" t="s">
         <v>48</v>
@@ -18796,7 +18796,7 @@
         <v>175</v>
       </c>
       <c r="C335" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D335" s="3" t="s">
         <v>20</v>
@@ -18838,7 +18838,7 @@
         <v>39</v>
       </c>
       <c r="C338" s="1" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D338" s="3" t="s">
         <v>48</v>
@@ -18853,7 +18853,7 @@
         <v>475</v>
       </c>
       <c r="C339" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D339" s="3" t="s">
         <v>20</v>
@@ -18910,7 +18910,7 @@
         <v>208</v>
       </c>
       <c r="C343" s="1" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D343" s="3" t="s">
         <v>20</v>
@@ -19050,7 +19050,7 @@
         <v>140</v>
       </c>
       <c r="C353" s="1" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D353" s="3" t="s">
         <v>48</v>
@@ -19064,7 +19064,7 @@
         <v>800</v>
       </c>
       <c r="C354" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="D354" s="3" t="s">
         <v>20</v>
@@ -19078,7 +19078,7 @@
         <v>830</v>
       </c>
       <c r="C355" s="1" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D355" s="3" t="s">
         <v>20</v>
@@ -19106,7 +19106,7 @@
         <v>325</v>
       </c>
       <c r="C357" s="1" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D357" s="3" t="s">
         <v>20</v>
@@ -19274,7 +19274,7 @@
         <v>60</v>
       </c>
       <c r="C369" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D369" s="3" t="s">
         <v>20</v>
@@ -19358,7 +19358,7 @@
         <v>150</v>
       </c>
       <c r="C375" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D375" s="3" t="s">
         <v>20</v>
@@ -19373,7 +19373,7 @@
         <v>296</v>
       </c>
       <c r="C376" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D376" s="3" t="s">
         <v>20</v>
@@ -19387,7 +19387,7 @@
         <v>80</v>
       </c>
       <c r="C377" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D377" s="3" t="s">
         <v>22</v>
@@ -19588,7 +19588,7 @@
         <v>1684</v>
       </c>
       <c r="C392" s="1" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D392" s="3" t="s">
         <v>20</v>
@@ -19630,7 +19630,7 @@
         <v>40</v>
       </c>
       <c r="C395" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D395" s="3" t="s">
         <v>48</v>
@@ -19733,7 +19733,7 @@
         <v>572</v>
       </c>
       <c r="C403" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D403" s="3" t="s">
         <v>20</v>
@@ -19747,7 +19747,7 @@
         <v>161</v>
       </c>
       <c r="C404" s="1" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D404" s="3" t="s">
         <v>20</v>
@@ -19761,7 +19761,7 @@
         <v>100</v>
       </c>
       <c r="C405" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D405" s="3" t="s">
         <v>388</v>
@@ -19887,7 +19887,7 @@
         <v>443</v>
       </c>
       <c r="C414" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="D414" s="3" t="s">
         <v>20</v>
@@ -19901,7 +19901,7 @@
         <v>443</v>
       </c>
       <c r="C415" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="D415" s="3" t="s">
         <v>20</v>
@@ -19915,7 +19915,7 @@
         <v>50</v>
       </c>
       <c r="C416" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D416" s="3" t="s">
         <v>20</v>
@@ -20007,7 +20007,7 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A423" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B423" s="1">
         <v>50</v>
@@ -20021,7 +20021,7 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A424" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B424" s="1">
         <v>25</v>
@@ -20035,14 +20035,14 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A425" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B425" s="1">
         <f>130+55+50</f>
         <v>235</v>
       </c>
       <c r="C425" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D425" s="3" t="s">
         <v>20</v>
@@ -20154,7 +20154,7 @@
         <v>160</v>
       </c>
       <c r="C433" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D433" s="3" t="s">
         <v>20</v>
@@ -20169,7 +20169,7 @@
         <v>300</v>
       </c>
       <c r="C434" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D434" s="3" t="s">
         <v>388</v>
@@ -20240,7 +20240,7 @@
         <v>154</v>
       </c>
       <c r="C439" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D439" s="3" t="s">
         <v>20</v>
@@ -20268,7 +20268,7 @@
         <v>75</v>
       </c>
       <c r="C441" s="1" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D441" s="3" t="s">
         <v>20</v>
@@ -20368,7 +20368,7 @@
         <v>658</v>
       </c>
       <c r="C448" s="1" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D448" s="3" t="s">
         <v>20</v>
@@ -21020,7 +21020,7 @@
         <v>1100</v>
       </c>
       <c r="C495" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D495" s="3" t="s">
         <v>20</v>
@@ -21034,7 +21034,7 @@
         <v>900</v>
       </c>
       <c r="C496" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D496" s="3" t="s">
         <v>20</v>
@@ -21165,7 +21165,7 @@
         <v>150</v>
       </c>
       <c r="C506" s="1" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D506" s="3" t="s">
         <v>395</v>
@@ -21201,7 +21201,7 @@
     </row>
     <row r="509" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A509" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B509" s="1">
         <v>20</v>
@@ -21215,7 +21215,7 @@
     </row>
     <row r="510" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A510" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="B510" s="1">
         <v>25</v>
@@ -21229,7 +21229,7 @@
     </row>
     <row r="511" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A511" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B511" s="1">
         <v>175</v>
@@ -21243,13 +21243,13 @@
     </row>
     <row r="512" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A512" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B512" s="1">
         <v>215</v>
       </c>
       <c r="C512" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D512" s="3" t="s">
         <v>20</v>
@@ -21257,7 +21257,7 @@
     </row>
     <row r="513" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A513" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B513" s="1">
         <v>150</v>
@@ -21271,7 +21271,7 @@
     </row>
     <row r="514" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A514" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B514" s="1">
         <v>60</v>
@@ -21285,7 +21285,7 @@
     </row>
     <row r="515" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A515" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B515" s="1">
         <v>350</v>
@@ -21306,7 +21306,7 @@
         <v>530</v>
       </c>
       <c r="C516" s="1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D516" s="3" t="s">
         <v>20</v>
@@ -21405,7 +21405,7 @@
         <v>285</v>
       </c>
       <c r="C523" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D523" s="3" t="s">
         <v>20</v>
@@ -21413,13 +21413,13 @@
     </row>
     <row r="524" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A524" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B524" s="1">
         <v>490</v>
       </c>
       <c r="C524" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D524" s="3" t="s">
         <v>20</v>
@@ -21427,13 +21427,13 @@
     </row>
     <row r="525" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A525" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B525" s="1">
         <v>5240</v>
       </c>
       <c r="C525" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D525" s="3" t="s">
         <v>20</v>
@@ -21441,13 +21441,13 @@
     </row>
     <row r="526" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A526" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B526" s="1">
         <v>6980</v>
       </c>
       <c r="C526" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D526" s="3" t="s">
         <v>20</v>
@@ -21455,7 +21455,7 @@
     </row>
     <row r="527" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A527" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B527" s="1">
         <v>40</v>
@@ -21469,13 +21469,13 @@
     </row>
     <row r="528" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A528" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B528" s="1">
         <v>195</v>
       </c>
       <c r="C528" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D528" s="3" t="s">
         <v>395</v>
@@ -21483,7 +21483,7 @@
     </row>
     <row r="529" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A529" s="1" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B529" s="1">
         <v>50</v>
@@ -21503,7 +21503,7 @@
         <v>105</v>
       </c>
       <c r="C530" s="1" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D530" s="3" t="s">
         <v>20</v>
@@ -21545,7 +21545,7 @@
         <v>60</v>
       </c>
       <c r="C533" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D533" s="3" t="s">
         <v>402</v>
@@ -21560,7 +21560,7 @@
         <v>165</v>
       </c>
       <c r="C534" s="1" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="D534" s="3" t="s">
         <v>395</v>
@@ -21610,13 +21610,13 @@
     </row>
     <row r="538" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A538" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B538" s="1">
         <v>95</v>
       </c>
       <c r="C538" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D538" s="3" t="s">
         <v>20</v>
@@ -21624,7 +21624,7 @@
     </row>
     <row r="539" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A539" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B539" s="1">
         <v>20</v>
@@ -21638,13 +21638,13 @@
     </row>
     <row r="540" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A540" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B540" s="1">
         <v>175</v>
       </c>
       <c r="C540" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D540" s="3" t="s">
         <v>20</v>
@@ -21658,7 +21658,7 @@
         <v>160</v>
       </c>
       <c r="C541" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="D541" s="3" t="s">
         <v>20</v>
@@ -21692,7 +21692,7 @@
         <v>868</v>
       </c>
       <c r="C544" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D544" s="3" t="s">
         <v>20</v>
@@ -21706,7 +21706,7 @@
         <v>80</v>
       </c>
       <c r="C545" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D545" s="3" t="s">
         <v>20</v>
@@ -21790,7 +21790,7 @@
         <v>60</v>
       </c>
       <c r="C551" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="D551" s="3" t="s">
         <v>395</v>
@@ -21846,7 +21846,7 @@
         <v>60</v>
       </c>
       <c r="C555" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D555" s="3" t="s">
         <v>20</v>
@@ -21959,7 +21959,7 @@
         <v>155</v>
       </c>
       <c r="C563" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D563" s="3" t="s">
         <v>20</v>
@@ -22015,7 +22015,7 @@
         <v>80</v>
       </c>
       <c r="C567" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D567" s="3" t="s">
         <v>20</v>
@@ -22114,7 +22114,7 @@
         <v>345</v>
       </c>
       <c r="C574" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D574" s="3" t="s">
         <v>35</v>
@@ -22198,7 +22198,7 @@
         <v>105</v>
       </c>
       <c r="C580" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D580" s="3" t="s">
         <v>35</v>
@@ -22381,7 +22381,7 @@
     </row>
     <row r="595" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A595" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B595" s="1">
         <v>16353</v>
@@ -22389,7 +22389,7 @@
     </row>
     <row r="596" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A596" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B596" s="1">
         <f>B593-B594-B595</f>

</xml_diff>

<commit_message>
Misc. Fixes + Tweaks - 2 typo fixes for the last commit (some Has rules weren't changed to HasAll) - Fixed the Icy Wilderness impossible start fix. It was inadvertently moved to be too early in generate_early to actually do its job. 	- It also accidentally wasn't even a fix...icy wilderness was being replaced with...icy wilderness lol. Whoops. - Progressive shop unlocks for starting realm levels (when pause menu patch is open shop) was being done in all sorts of ways wrong. 	- Now, the correct amount of progressive/reverse progressive shop unlocks are given in start inventory, and the rest are in the item pool. - Decluttered/reworded parts of the log system. 	- Removed a few redundant "checking for x" messages 	- Added info about where each created item is being placed. 	- The log message for random boss choices was a bit misleading.
</commit_message>
<xml_diff>
--- a/worlds/spyro_aht/setup/Gem Research.xlsx
+++ b/worlds/spyro_aht/setup/Gem Research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAE3FBF1-E438-40C5-90BC-5279D589720C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B4B889-6C5B-4C9F-85D9-730BC5B7D71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2348,7 +2348,7 @@
     <t>HasAll('Double Jump', 'Fire Breath', 'Electric Breath')</t>
   </si>
   <si>
-    <t>Has('Double Jump', 'Electric Breath')</t>
+    <t>HasAll('Double Jump', 'Electric Breath')</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fixed Logic Issue with RLSouthEast1 - It only required charge even though armored middle robo-gnorcs also require (electric or ice). - Also condensed 2 gem rules in the southeast area. One was missed months ago, one was enabled by this fix.
</commit_message>
<xml_diff>
--- a/worlds/spyro_aht/setup/Gem Research.xlsx
+++ b/worlds/spyro_aht/setup/Gem Research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sean\Downloads\Archipelago Stuff\apworlds\PhoenixAP\worlds\spyro_aht\setup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58B4B889-6C5B-4C9F-85D9-730BC5B7D71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C7FBA1-1679-4DFF-9516-8139E5B0F352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="697" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -297,7 +297,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4186" uniqueCount="684">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4180" uniqueCount="686">
   <si>
     <t>DVEntry</t>
   </si>
@@ -2186,9 +2186,6 @@
     <t>metal chests/headbash chests/and baskets using DJ</t>
   </si>
   <si>
-    <t>baskets behind lasers/headbash chest</t>
-  </si>
-  <si>
     <t>NON-BLINK ENEMIES</t>
   </si>
   <si>
@@ -2349,6 +2346,15 @@
   </si>
   <si>
     <t>HasAll('Double Jump', 'Electric Breath')</t>
+  </si>
+  <si>
+    <t>[enemy] armored middle robo-gnorc and small robo-gnorc</t>
+  </si>
+  <si>
+    <t>baskets behind lasers + headbash chest</t>
+  </si>
+  <si>
+    <t>[enemy] armored middle robo-gnorc + huge robo-gnorcs up high</t>
   </si>
 </sst>
 </file>
@@ -2715,7 +2721,7 @@
   <cols>
     <col min="1" max="1" width="41.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="98" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="107.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="170.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="115.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -2927,7 +2933,7 @@
         <v>395</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>20</v>
@@ -2941,7 +2947,7 @@
         <v>360</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>20</v>
@@ -3941,7 +3947,7 @@
         <v>1003</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>20</v>
@@ -3955,7 +3961,7 @@
         <v>928</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>20</v>
@@ -4436,7 +4442,7 @@
         <v>675</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>20</v>
@@ -4450,7 +4456,7 @@
         <v>700</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>20</v>
@@ -5834,7 +5840,7 @@
         <v>755</v>
       </c>
       <c r="C223" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D223" s="3" t="s">
         <v>20</v>
@@ -5848,7 +5854,7 @@
         <v>1435</v>
       </c>
       <c r="C224" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D224" s="3" t="s">
         <v>20</v>
@@ -6651,7 +6657,7 @@
         <v>200</v>
       </c>
       <c r="C282" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D282" s="3" t="s">
         <v>20</v>
@@ -6665,7 +6671,7 @@
         <v>200</v>
       </c>
       <c r="C283" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D283" s="3" t="s">
         <v>20</v>
@@ -7272,7 +7278,7 @@
         <v>900</v>
       </c>
       <c r="C327" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D327" s="3" t="s">
         <v>20</v>
@@ -7286,7 +7292,7 @@
         <v>800</v>
       </c>
       <c r="C328" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D328" s="3" t="s">
         <v>20</v>
@@ -7710,7 +7716,7 @@
         <v>194</v>
       </c>
       <c r="D358" s="3" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.45">
@@ -7721,10 +7727,10 @@
         <v>50</v>
       </c>
       <c r="C359" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D359" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.45">
@@ -7735,7 +7741,7 @@
         <v>100</v>
       </c>
       <c r="C360" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D360" s="3" t="s">
         <v>209</v>
@@ -8118,7 +8124,7 @@
         <v>1906</v>
       </c>
       <c r="C388" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D388" s="3" t="s">
         <v>20</v>
@@ -8132,7 +8138,7 @@
         <v>1956</v>
       </c>
       <c r="C389" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D389" s="3" t="s">
         <v>20</v>
@@ -8205,7 +8211,7 @@
         <v>50</v>
       </c>
       <c r="C394" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D394" s="3" t="s">
         <v>211</v>
@@ -8891,7 +8897,7 @@
     </row>
     <row r="444" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A444" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B444" s="1">
         <v>110</v>
@@ -8905,7 +8911,7 @@
     </row>
     <row r="445" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A445" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B445" s="1">
         <v>156</v>
@@ -8922,7 +8928,7 @@
     </row>
     <row r="446" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A446" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B446" s="1">
         <v>400</v>
@@ -8936,7 +8942,7 @@
     </row>
     <row r="447" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A447" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B447" s="1">
         <v>500</v>
@@ -8950,7 +8956,7 @@
     </row>
     <row r="448" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A448" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B448" s="1">
         <v>400</v>
@@ -8964,7 +8970,7 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A449" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B449" s="1">
         <v>60</v>
@@ -8978,7 +8984,7 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A450" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B450" s="1">
         <v>100</v>
@@ -8992,7 +8998,7 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A451" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B451" s="1">
         <v>1000</v>
@@ -9006,7 +9012,7 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A452" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B452" s="1">
         <v>450</v>
@@ -9020,7 +9026,7 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A453" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B453" s="1">
         <v>50</v>
@@ -9034,13 +9040,13 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A454" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B454" s="1">
         <v>950</v>
       </c>
       <c r="C454" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D454" s="3" t="s">
         <v>20</v>
@@ -9048,13 +9054,13 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A455" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B455" s="1">
         <v>900</v>
       </c>
       <c r="C455" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D455" s="3" t="s">
         <v>20</v>
@@ -9062,7 +9068,7 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A456" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B456" s="1">
         <v>200</v>
@@ -9689,7 +9695,7 @@
         <v>800</v>
       </c>
       <c r="C501" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D501" s="3" t="s">
         <v>20</v>
@@ -9703,7 +9709,7 @@
         <v>830</v>
       </c>
       <c r="C502" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D502" s="3" t="s">
         <v>20</v>
@@ -10369,7 +10375,7 @@
         <v>270</v>
       </c>
       <c r="C550" s="1" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="D550" s="3" t="s">
         <v>20</v>
@@ -10794,7 +10800,7 @@
         <v>443</v>
       </c>
       <c r="C581" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D581" s="3" t="s">
         <v>20</v>
@@ -10808,7 +10814,7 @@
         <v>443</v>
       </c>
       <c r="C582" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D582" s="3" t="s">
         <v>20</v>
@@ -10822,7 +10828,7 @@
         <v>50</v>
       </c>
       <c r="C583" s="1" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D583" s="3" t="s">
         <v>20</v>
@@ -10914,13 +10920,13 @@
     </row>
     <row r="590" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A590" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B590" s="1">
         <v>50</v>
       </c>
       <c r="C590" s="1" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="D590" s="3" t="s">
         <v>20</v>
@@ -10928,7 +10934,7 @@
     </row>
     <row r="591" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A591" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B591" s="1">
         <v>25</v>
@@ -10942,7 +10948,7 @@
     </row>
     <row r="592" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A592" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B592" s="1">
         <v>130</v>
@@ -10956,7 +10962,7 @@
     </row>
     <row r="593" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A593" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B593" s="1">
         <v>55</v>
@@ -10970,7 +10976,7 @@
     </row>
     <row r="594" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A594" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B594" s="1">
         <v>50</v>
@@ -12202,7 +12208,7 @@
         <v>1100</v>
       </c>
       <c r="C682" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D682" s="3" t="s">
         <v>20</v>
@@ -12216,7 +12222,7 @@
         <v>900</v>
       </c>
       <c r="C683" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D683" s="3" t="s">
         <v>20</v>
@@ -12411,7 +12417,7 @@
     </row>
     <row r="698" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A698" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B698" s="1">
         <v>20</v>
@@ -12425,7 +12431,7 @@
     </row>
     <row r="699" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A699" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B699" s="1">
         <v>25</v>
@@ -12439,7 +12445,7 @@
     </row>
     <row r="700" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A700" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B700" s="1">
         <v>100</v>
@@ -12453,7 +12459,7 @@
     </row>
     <row r="701" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A701" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B701" s="1">
         <v>75</v>
@@ -12467,7 +12473,7 @@
     </row>
     <row r="702" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A702" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B702" s="1">
         <v>40</v>
@@ -12481,7 +12487,7 @@
     </row>
     <row r="703" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A703" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B703" s="1">
         <v>150</v>
@@ -12495,7 +12501,7 @@
     </row>
     <row r="704" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A704" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B704" s="1">
         <v>125</v>
@@ -12509,7 +12515,7 @@
     </row>
     <row r="705" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A705" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B705" s="1">
         <v>60</v>
@@ -12523,7 +12529,7 @@
     </row>
     <row r="706" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A706" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B706" s="1">
         <v>50</v>
@@ -12537,7 +12543,7 @@
     </row>
     <row r="707" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A707" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B707" s="1">
         <v>350</v>
@@ -12750,7 +12756,7 @@
     </row>
     <row r="722" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A722" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B722" s="1">
         <v>200</v>
@@ -12764,7 +12770,7 @@
     </row>
     <row r="723" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A723" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B723" s="1">
         <v>100</v>
@@ -12778,7 +12784,7 @@
     </row>
     <row r="724" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A724" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B724" s="1">
         <v>100</v>
@@ -12792,7 +12798,7 @@
     </row>
     <row r="725" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A725" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B725" s="1">
         <v>90</v>
@@ -12806,13 +12812,13 @@
     </row>
     <row r="726" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A726" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B726" s="1">
         <v>5240</v>
       </c>
       <c r="C726" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D726" s="3" t="s">
         <v>20</v>
@@ -12820,13 +12826,13 @@
     </row>
     <row r="727" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A727" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B727" s="1">
         <v>6980</v>
       </c>
       <c r="C727" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D727" s="3" t="s">
         <v>20</v>
@@ -12834,7 +12840,7 @@
     </row>
     <row r="728" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A728" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B728" s="1">
         <v>40</v>
@@ -12848,7 +12854,7 @@
     </row>
     <row r="729" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A729" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B729" s="1">
         <v>175</v>
@@ -12862,13 +12868,13 @@
     </row>
     <row r="730" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A730" s="1" t="s">
+        <v>662</v>
+      </c>
+      <c r="B730" s="1">
+        <v>20</v>
+      </c>
+      <c r="C730" s="1" t="s">
         <v>663</v>
-      </c>
-      <c r="B730" s="1">
-        <v>20</v>
-      </c>
-      <c r="C730" s="1" t="s">
-        <v>664</v>
       </c>
       <c r="D730" s="3" t="s">
         <v>392</v>
@@ -12876,7 +12882,7 @@
     </row>
     <row r="731" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A731" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B731" s="1">
         <v>50</v>
@@ -13058,7 +13064,7 @@
     </row>
     <row r="744" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A744" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B744" s="1">
         <v>75</v>
@@ -13072,7 +13078,7 @@
     </row>
     <row r="745" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A745" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B745" s="1">
         <v>20</v>
@@ -13086,7 +13092,7 @@
     </row>
     <row r="746" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A746" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B746" s="1">
         <v>20</v>
@@ -13100,7 +13106,7 @@
     </row>
     <row r="747" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A747" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B747" s="1">
         <v>50</v>
@@ -13114,7 +13120,7 @@
     </row>
     <row r="748" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A748" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B748" s="1">
         <v>100</v>
@@ -13128,7 +13134,7 @@
     </row>
     <row r="749" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A749" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B749" s="1">
         <v>25</v>
@@ -13884,7 +13890,7 @@
         <v>510</v>
       </c>
       <c r="D803" s="3" t="s">
-        <v>393</v>
+        <v>20</v>
       </c>
     </row>
     <row r="804" spans="1:4" x14ac:dyDescent="0.45">
@@ -13968,7 +13974,7 @@
         <v>524</v>
       </c>
       <c r="D809" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="810" spans="1:4" x14ac:dyDescent="0.45">
@@ -14116,7 +14122,7 @@
     </row>
     <row r="822" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A822" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B822" s="1">
         <v>16353</v>
@@ -14124,7 +14130,7 @@
     </row>
     <row r="823" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A823" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B823" s="1">
         <f>B820-B821-B822</f>
@@ -14140,7 +14146,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABB84367-A097-4248-9984-F4697DA02168}">
-  <dimension ref="A1:D595"/>
+  <dimension ref="A1:D593"/>
   <sheetFormatPr defaultRowHeight="28.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="41.140625" style="1" bestFit="1" customWidth="1"/>
@@ -14276,7 +14282,7 @@
         <v>395</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>20</v>
@@ -14290,7 +14296,7 @@
         <v>360</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>20</v>
@@ -15000,7 +15006,7 @@
         <v>1003</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>20</v>
@@ -15014,7 +15020,7 @@
         <v>928</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>20</v>
@@ -15358,7 +15364,7 @@
         <v>675</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>20</v>
@@ -15372,7 +15378,7 @@
         <v>700</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>20</v>
@@ -16109,7 +16115,7 @@
         <v>525</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>20</v>
@@ -16376,7 +16382,7 @@
         <v>755</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>20</v>
@@ -16390,7 +16396,7 @@
         <v>1435</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>20</v>
@@ -16875,7 +16881,7 @@
         <v>200</v>
       </c>
       <c r="C197" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D197" s="3" t="s">
         <v>20</v>
@@ -16889,7 +16895,7 @@
         <v>200</v>
       </c>
       <c r="C198" s="1" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>20</v>
@@ -16918,7 +16924,7 @@
         <v>410</v>
       </c>
       <c r="C200" s="1" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="D200" s="3" t="s">
         <v>20</v>
@@ -17373,7 +17379,7 @@
         <v>900</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="D233" s="3" t="s">
         <v>20</v>
@@ -17387,7 +17393,7 @@
         <v>800</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="D234" s="3" t="s">
         <v>20</v>
@@ -17515,7 +17521,7 @@
         <v>606</v>
       </c>
       <c r="C243" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D243" s="3" t="s">
         <v>20</v>
@@ -17543,7 +17549,7 @@
         <v>235</v>
       </c>
       <c r="C245" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D245" s="3" t="s">
         <v>20</v>
@@ -17645,7 +17651,7 @@
         <v>194</v>
       </c>
       <c r="D252" s="3" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.45">
@@ -17656,10 +17662,10 @@
         <v>50</v>
       </c>
       <c r="C253" s="1" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="D253" s="3" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.45">
@@ -17670,7 +17676,7 @@
         <v>100</v>
       </c>
       <c r="C254" s="1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D254" s="3" t="s">
         <v>209</v>
@@ -17888,7 +17894,7 @@
         <v>1906</v>
       </c>
       <c r="C270" s="1" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D270" s="3" t="s">
         <v>20</v>
@@ -17902,7 +17908,7 @@
         <v>1956</v>
       </c>
       <c r="C271" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D271" s="3" t="s">
         <v>20</v>
@@ -17958,7 +17964,7 @@
         <v>50</v>
       </c>
       <c r="C275" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D275" s="3" t="s">
         <v>211</v>
@@ -18028,7 +18034,7 @@
         <v>141</v>
       </c>
       <c r="C280" s="1" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="D280" s="3" t="s">
         <v>22</v>
@@ -18463,7 +18469,7 @@
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A312" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B312" s="1">
         <v>110</v>
@@ -18477,7 +18483,7 @@
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A313" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B313" s="1">
         <v>656</v>
@@ -18491,7 +18497,7 @@
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A314" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B314" s="1">
         <v>1060</v>
@@ -18505,7 +18511,7 @@
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A315" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B315" s="1">
         <v>400</v>
@@ -18519,7 +18525,7 @@
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A316" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B316" s="1">
         <v>1000</v>
@@ -18533,13 +18539,13 @@
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A317" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B317" s="1">
         <v>200</v>
       </c>
       <c r="C317" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D317" s="3" t="s">
         <v>20</v>
@@ -18547,13 +18553,13 @@
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A318" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B318" s="1">
         <v>950</v>
       </c>
       <c r="C318" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="D318" s="3" t="s">
         <v>20</v>
@@ -18561,13 +18567,13 @@
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A319" s="1" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B319" s="1">
         <v>900</v>
       </c>
       <c r="C319" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D319" s="3" t="s">
         <v>20</v>
@@ -19036,7 +19042,7 @@
         <v>800</v>
       </c>
       <c r="C353" s="1" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D353" s="3" t="s">
         <v>20</v>
@@ -19050,7 +19056,7 @@
         <v>830</v>
       </c>
       <c r="C354" s="1" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D354" s="3" t="s">
         <v>20</v>
@@ -19859,7 +19865,7 @@
         <v>443</v>
       </c>
       <c r="C413" s="1" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="D413" s="3" t="s">
         <v>20</v>
@@ -19873,7 +19879,7 @@
         <v>443</v>
       </c>
       <c r="C414" s="1" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="D414" s="3" t="s">
         <v>20</v>
@@ -19887,7 +19893,7 @@
         <v>50</v>
       </c>
       <c r="C415" s="1" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="D415" s="3" t="s">
         <v>20</v>
@@ -19979,7 +19985,7 @@
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A422" s="1" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="B422" s="1">
         <v>50</v>
@@ -19993,7 +19999,7 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A423" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B423" s="1">
         <v>25</v>
@@ -20007,7 +20013,7 @@
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A424" s="1" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B424" s="1">
         <f>130+55+50</f>
@@ -20992,7 +20998,7 @@
         <v>1100</v>
       </c>
       <c r="C494" s="1" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="D494" s="3" t="s">
         <v>20</v>
@@ -21006,7 +21012,7 @@
         <v>900</v>
       </c>
       <c r="C495" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="D495" s="3" t="s">
         <v>20</v>
@@ -21173,7 +21179,7 @@
     </row>
     <row r="508" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A508" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B508" s="1">
         <v>20</v>
@@ -21187,7 +21193,7 @@
     </row>
     <row r="509" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A509" s="1" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="B509" s="1">
         <v>25</v>
@@ -21201,7 +21207,7 @@
     </row>
     <row r="510" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A510" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B510" s="1">
         <v>175</v>
@@ -21215,13 +21221,13 @@
     </row>
     <row r="511" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A511" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B511" s="1">
         <v>215</v>
       </c>
       <c r="C511" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="D511" s="3" t="s">
         <v>20</v>
@@ -21229,7 +21235,7 @@
     </row>
     <row r="512" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A512" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B512" s="1">
         <v>150</v>
@@ -21243,7 +21249,7 @@
     </row>
     <row r="513" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A513" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B513" s="1">
         <v>60</v>
@@ -21257,7 +21263,7 @@
     </row>
     <row r="514" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A514" s="1" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="B514" s="1">
         <v>350</v>
@@ -21385,7 +21391,7 @@
     </row>
     <row r="523" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A523" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B523" s="1">
         <v>490</v>
@@ -21399,13 +21405,13 @@
     </row>
     <row r="524" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A524" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B524" s="1">
         <v>5240</v>
       </c>
       <c r="C524" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D524" s="3" t="s">
         <v>20</v>
@@ -21413,13 +21419,13 @@
     </row>
     <row r="525" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A525" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B525" s="1">
         <v>6980</v>
       </c>
       <c r="C525" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D525" s="3" t="s">
         <v>20</v>
@@ -21427,7 +21433,7 @@
     </row>
     <row r="526" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A526" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B526" s="1">
         <v>40</v>
@@ -21441,13 +21447,13 @@
     </row>
     <row r="527" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A527" s="1" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B527" s="1">
         <v>195</v>
       </c>
       <c r="C527" s="1" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="D527" s="3" t="s">
         <v>392</v>
@@ -21455,7 +21461,7 @@
     </row>
     <row r="528" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A528" s="1" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B528" s="1">
         <v>50</v>
@@ -21517,7 +21523,7 @@
         <v>60</v>
       </c>
       <c r="C532" s="1" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="D532" s="3" t="s">
         <v>399</v>
@@ -21532,7 +21538,7 @@
         <v>165</v>
       </c>
       <c r="C533" s="1" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="D533" s="3" t="s">
         <v>392</v>
@@ -21582,13 +21588,13 @@
     </row>
     <row r="537" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A537" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B537" s="1">
         <v>95</v>
       </c>
       <c r="C537" s="1" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="D537" s="3" t="s">
         <v>20</v>
@@ -21596,7 +21602,7 @@
     </row>
     <row r="538" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A538" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B538" s="1">
         <v>20</v>
@@ -21610,7 +21616,7 @@
     </row>
     <row r="539" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A539" s="1" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="B539" s="1">
         <v>175</v>
@@ -22125,13 +22131,13 @@
         <v>377</v>
       </c>
       <c r="B576" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C576" s="1" t="s">
-        <v>510</v>
+        <v>683</v>
       </c>
       <c r="D576" s="3" t="s">
-        <v>393</v>
+        <v>20</v>
       </c>
     </row>
     <row r="577" spans="1:4" x14ac:dyDescent="0.45">
@@ -22139,10 +22145,10 @@
         <v>377</v>
       </c>
       <c r="B577" s="1">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C577" s="1" t="s">
-        <v>507</v>
+        <v>24</v>
       </c>
       <c r="D577" s="3" t="s">
         <v>20</v>
@@ -22153,27 +22159,27 @@
         <v>377</v>
       </c>
       <c r="B578" s="1">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="C578" s="1" t="s">
-        <v>24</v>
+        <v>684</v>
       </c>
       <c r="D578" s="3" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="579" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A579" s="1" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B579" s="1">
-        <v>105</v>
+        <v>75</v>
       </c>
       <c r="C579" s="1" t="s">
-        <v>629</v>
+        <v>378</v>
       </c>
       <c r="D579" s="3" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
     </row>
     <row r="580" spans="1:4" x14ac:dyDescent="0.45">
@@ -22181,10 +22187,10 @@
         <v>379</v>
       </c>
       <c r="B580" s="1">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C580" s="1" t="s">
-        <v>378</v>
+        <v>685</v>
       </c>
       <c r="D580" s="3" t="s">
         <v>20</v>
@@ -22192,30 +22198,30 @@
     </row>
     <row r="581" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A581" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B581" s="1">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C581" s="1" t="s">
-        <v>524</v>
+        <v>510</v>
       </c>
       <c r="D581" s="3" t="s">
-        <v>22</v>
+        <v>402</v>
       </c>
     </row>
     <row r="582" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A582" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B582" s="1">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C582" s="1" t="s">
-        <v>525</v>
+        <v>517</v>
       </c>
       <c r="D582" s="3" t="s">
-        <v>20</v>
+        <v>399</v>
       </c>
     </row>
     <row r="583" spans="1:4" x14ac:dyDescent="0.45">
@@ -22223,13 +22229,13 @@
         <v>380</v>
       </c>
       <c r="B583" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C583" s="1" t="s">
-        <v>510</v>
+        <v>33</v>
       </c>
       <c r="D583" s="3" t="s">
-        <v>402</v>
+        <v>35</v>
       </c>
     </row>
     <row r="584" spans="1:4" x14ac:dyDescent="0.45">
@@ -22237,13 +22243,13 @@
         <v>380</v>
       </c>
       <c r="B584" s="1">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C584" s="1" t="s">
-        <v>517</v>
+        <v>24</v>
       </c>
       <c r="D584" s="3" t="s">
-        <v>399</v>
+        <v>27</v>
       </c>
     </row>
     <row r="585" spans="1:4" x14ac:dyDescent="0.45">
@@ -22251,13 +22257,13 @@
         <v>380</v>
       </c>
       <c r="B585" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C585" s="1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D585" s="3" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="586" spans="1:4" x14ac:dyDescent="0.45">
@@ -22265,13 +22271,13 @@
         <v>380</v>
       </c>
       <c r="B586" s="1">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="C586" s="1" t="s">
-        <v>24</v>
+        <v>506</v>
       </c>
       <c r="D586" s="3" t="s">
-        <v>27</v>
+        <v>392</v>
       </c>
     </row>
     <row r="587" spans="1:4" x14ac:dyDescent="0.45">
@@ -22282,10 +22288,10 @@
         <v>50</v>
       </c>
       <c r="C587" s="1" t="s">
-        <v>23</v>
+        <v>381</v>
       </c>
       <c r="D587" s="3" t="s">
-        <v>26</v>
+        <v>398</v>
       </c>
     </row>
     <row r="588" spans="1:4" x14ac:dyDescent="0.45">
@@ -22296,78 +22302,50 @@
         <v>20</v>
       </c>
       <c r="C588" s="1" t="s">
-        <v>506</v>
+        <v>526</v>
       </c>
       <c r="D588" s="3" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="589" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A589" s="1" t="s">
-        <v>380</v>
-      </c>
-      <c r="B589" s="1">
-        <v>50</v>
-      </c>
-      <c r="C589" s="1" t="s">
-        <v>381</v>
-      </c>
-      <c r="D589" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="590" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A590" s="1" t="s">
-        <v>380</v>
+        <v>407</v>
       </c>
       <c r="B590" s="1">
-        <v>20</v>
-      </c>
-      <c r="C590" s="1" t="s">
-        <v>526</v>
-      </c>
-      <c r="D590" s="3" t="s">
-        <v>401</v>
+        <f>SUM(B2:B588)</f>
+        <v>141913</v>
+      </c>
+      <c r="C590" s="1" t="str">
+        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B820</f>
+        <v>should be 141913</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A591" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B591" s="1">
+        <v>20203</v>
       </c>
     </row>
     <row r="592" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A592" s="1" t="s">
-        <v>407</v>
+        <v>629</v>
       </c>
       <c r="B592" s="1">
-        <f>SUM(B2:B590)</f>
-        <v>141913</v>
-      </c>
-      <c r="C592" s="1" t="str">
-        <f>"should be " &amp; 'New Gems (simplified per-rule)'!B820</f>
-        <v>should be 141913</v>
+        <v>16353</v>
       </c>
     </row>
     <row r="593" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A593" s="1" t="s">
-        <v>17</v>
+        <v>630</v>
       </c>
       <c r="B593" s="1">
-        <v>20203</v>
-      </c>
-    </row>
-    <row r="594" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A594" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="B594" s="1">
-        <v>16353</v>
-      </c>
-    </row>
-    <row r="595" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A595" s="1" t="s">
-        <v>631</v>
-      </c>
-      <c r="B595" s="1">
-        <f>B592-B593-B594</f>
+        <f>B590-B591-B592</f>
         <v>105357</v>
       </c>
-      <c r="C595" s="1" t="str">
+      <c r="C593" s="1" t="str">
         <f>"should be " &amp; 'New Gems (simplified per-rule)'!B823</f>
         <v>should be 105357</v>
       </c>

</xml_diff>